<commit_message>
updated code chunk to include abundance data successfully
</commit_message>
<xml_diff>
--- a/Taxonomy_list_fermented_food_periodic_table.xlsx
+++ b/Taxonomy_list_fermented_food_periodic_table.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xinzhao/DS_Projects/phylo-tree-fermented-foods/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E2E51E4-A2E1-8B4A-BF63-E68A01054B0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{325F09F9-28B9-9247-B071-4FE40D4B5D95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4280" yWindow="760" windowWidth="25960" windowHeight="18880" activeTab="3" xr2:uid="{D834C665-731C-7E47-A8BF-B2F00BB8B4D6}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" activeTab="1" xr2:uid="{D834C665-731C-7E47-A8BF-B2F00BB8B4D6}"/>
   </bookViews>
   <sheets>
     <sheet name="extracted taxonomy" sheetId="3" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="802" uniqueCount="223">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="801" uniqueCount="222">
   <si>
     <t xml:space="preserve">Lactobacillaceae  </t>
   </si>
@@ -705,9 +705,6 @@
   </si>
   <si>
     <t>Fermented foods1</t>
-  </si>
-  <si>
-    <t>Fermented foods2</t>
   </si>
   <si>
     <t>Species</t>
@@ -889,7 +886,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4019,7 +4016,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{933E687C-0B8B-8446-9F3B-17B50211A94B}">
-  <dimension ref="A1:AK3"/>
+  <dimension ref="A1:AK2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15.83203125" customWidth="1"/>
@@ -4248,119 +4245,6 @@
         <v>7</v>
       </c>
       <c r="AK2">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="3" spans="1:37" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>221</v>
-      </c>
-      <c r="B3">
-        <v>16</v>
-      </c>
-      <c r="C3">
-        <v>16</v>
-      </c>
-      <c r="D3">
-        <v>16</v>
-      </c>
-      <c r="E3">
-        <v>3</v>
-      </c>
-      <c r="F3">
-        <v>16</v>
-      </c>
-      <c r="G3">
-        <v>16</v>
-      </c>
-      <c r="H3">
-        <v>16</v>
-      </c>
-      <c r="I3">
-        <v>16</v>
-      </c>
-      <c r="J3">
-        <v>101</v>
-      </c>
-      <c r="K3">
-        <v>101</v>
-      </c>
-      <c r="L3">
-        <v>101</v>
-      </c>
-      <c r="M3">
-        <v>101</v>
-      </c>
-      <c r="N3">
-        <v>101</v>
-      </c>
-      <c r="O3">
-        <v>101</v>
-      </c>
-      <c r="P3">
-        <v>101</v>
-      </c>
-      <c r="Q3">
-        <v>101</v>
-      </c>
-      <c r="R3">
-        <v>101</v>
-      </c>
-      <c r="S3">
-        <v>101</v>
-      </c>
-      <c r="T3">
-        <v>101</v>
-      </c>
-      <c r="U3">
-        <v>101</v>
-      </c>
-      <c r="V3">
-        <v>101</v>
-      </c>
-      <c r="W3">
-        <v>101</v>
-      </c>
-      <c r="X3">
-        <v>101</v>
-      </c>
-      <c r="Y3">
-        <v>101</v>
-      </c>
-      <c r="Z3">
-        <v>101</v>
-      </c>
-      <c r="AA3">
-        <v>101</v>
-      </c>
-      <c r="AB3">
-        <v>101</v>
-      </c>
-      <c r="AC3">
-        <v>101</v>
-      </c>
-      <c r="AD3">
-        <v>101</v>
-      </c>
-      <c r="AE3">
-        <v>101</v>
-      </c>
-      <c r="AF3">
-        <v>101</v>
-      </c>
-      <c r="AG3">
-        <v>9</v>
-      </c>
-      <c r="AH3">
-        <v>9</v>
-      </c>
-      <c r="AI3">
-        <v>1</v>
-      </c>
-      <c r="AJ3">
-        <v>7</v>
-      </c>
-      <c r="AK3">
         <v>7</v>
       </c>
     </row>
@@ -4407,7 +4291,7 @@
         <v>150</v>
       </c>
       <c r="H1" s="12" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="17" thickTop="1" x14ac:dyDescent="0.2">

</xml_diff>